<commit_message>
DM: VBC com ou sem d/y/t conforme incluir_vplbc; media por componente
- if/else por linha: incluir_vplbc = Sim aplica d, y e t no VBC; Nao
  calcula o VBC sem os parametros
- DM medio agrupado so por componente, com todas as linhas
- Nova funcao corrigir_numero() em R/DM-Corrigir_Numeros.R para
  numeros digitados como texto (ex.: "0,0317")

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01921tobnuBi7DJeDNAR5WiS
</commit_message>
<xml_diff>
--- a/Modelos/Entrada_DM.xlsx
+++ b/Modelos/Entrada_DM.xlsx
@@ -100,7 +100,7 @@
             <color rgb="FF000000"/>
             <name val="Tahoma"/>
           </rPr>
-          <t xml:space="preserve">Sim = entra no DM médio do componente; Não = fica de fora</t>
+          <t xml:space="preserve">Sim = VBC com os parâmetros d, y e t; Não = VBC sem os parâmetros</t>
         </r>
       </text>
     </comment>
@@ -205,7 +205,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="102">
   <si>
     <t xml:space="preserve">Planilha de entrada para R/DM-Calculo_Perdas_Ganhos.R</t>
   </si>
@@ -508,6 +508,9 @@
   </si>
   <si>
     <t xml:space="preserve">alta</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sim = VBC com os parâmetros d, y e t; Não = VBC sem os parâmetros</t>
   </si>
 </sst>
 </file>
@@ -1021,7 +1024,7 @@
         <v>12</v>
       </c>
       <c r="C16" t="s">
-        <v>31</v>
+        <v>101</v>
       </c>
       <c r="D16" t="s">
         <v>1</v>

</xml_diff>